<commit_message>
docs(v19): finalize approved canonical release metadata
Record PR73 approval and content merge, align distribution labels, preserve all ticket properties and WBS calculations, and rebuild manifest/checksums. Publication remains pending independent finalization review and actual Tag/Asset verification.
</commit_message>
<xml_diff>
--- a/wbs/FDS_v3.1.19_WBS_and_Gantt_v1.0.xlsx
+++ b/wbs/FDS_v3.1.19_WBS_and_Gantt_v1.0.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rfae9835becb8450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rcc138e90d38c4223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Rece9c63eb99b474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rb23053566ea54a1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R4409eae8f3b14581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R36c7a497fcca41ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R3c0be833ae7743ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Ra9d7cdee84c44778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R31109ef89c3b475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R235d9a4420af41c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R59ab6afb04f641c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R6acc04048ad9454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R2dbf830d11464908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Re2edcc124f574a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R8d9010e88a214b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R2a560c9bcc414f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R328307bbac4e4bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R64c4e033e0fb43bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -700,7 +700,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="45">
+  <x:dxfs count="50">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1080,6 +1080,41 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDF4EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF3CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FF3AB588"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDF4EA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF3CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFDDF4EA"/>
         </x:patternFill>
@@ -1363,7 +1398,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbba3d9ef1e2e4be3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R03ec23ce1b674b82"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1393,7 +1428,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0758e9560ba64ee1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ffaebfb66a04418"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1651,7 +1686,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Executive Schedule Summary (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Executive Schedule Summary (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -1712,7 +1747,7 @@
         <x:v>Canonical version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>3.1.19 CANDIDATE</x:v>
+        <x:v>3.1.19 RELEASED</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
         <x:v>G1 Target</x:v>
@@ -2085,7 +2120,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c7c1f5aa66d47de"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11db9abe047644f2"/>
 </x:worksheet>
 </file>
 
@@ -2116,7 +2151,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · WBS (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · WBS (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -5823,8 +5858,8 @@
     <x:cfRule type="containsText" dxfId="28" priority="12" operator="containsText" text="End TBD"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G59:G61">
-    <x:cfRule type="containsText" dxfId="40" priority="13" operator="containsText" text="Done"/>
-    <x:cfRule type="containsText" dxfId="41" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="45" priority="13" operator="containsText" text="Done"/>
+    <x:cfRule type="containsText" dxfId="46" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="G4:G54">
@@ -5845,7 +5880,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c29d88d53994675"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0d7c5dee9344273"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5893,7 +5928,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Phase 1 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Phase 1 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -10009,13 +10044,13 @@
     <x:cfRule type="containsText" dxfId="34" priority="14" operator="containsText" text="In Review"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G35:AI37">
-    <x:cfRule type="cellIs" dxfId="42" priority="17" operator="equal">
+    <x:cfRule type="cellIs" dxfId="47" priority="20" operator="equal">
       <x:formula>1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C35:C37">
-    <x:cfRule type="containsText" dxfId="43" priority="18" operator="containsText" text="Done"/>
-    <x:cfRule type="containsText" dxfId="44" priority="19" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="48" priority="21" operator="containsText" text="Done"/>
+    <x:cfRule type="containsText" dxfId="49" priority="22" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10064,7 +10099,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Phase 2 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Phase 2 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -13208,7 +13243,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Milestones &amp; Decision Calendar (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Milestones &amp; Decision Calendar (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -14294,7 +14329,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Risks, Assumptions &amp; Lead Decisions (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Risks, Assumptions &amp; Lead Decisions (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -14643,7 +14678,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Sources &amp; Change Log (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Sources &amp; Change Log (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -14688,19 +14723,19 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="str">
-        <x:v>Canonical candidate</x:v>
+        <x:v>Canonical baseline</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
         <x:v>FDS_Project_Implementation_Baseline_v3.1.19.md</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
-        <x:v>v3.1.19 CANDIDATE</x:v>
+        <x:v>v3.1.19 RELEASED</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="E4" s="13" t="str">
-        <x:v>Current candidate scope / release review pending</x:v>
+        <x:v>Approved content; finalization metadata subject to review/merge</x:v>
       </x:c>
       <x:c r="G4" s="13" t="str">
         <x:v>D36 / Team availability</x:v>
@@ -14714,7 +14749,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="13" t="str">
-        <x:v>Canonical candidate</x:v>
+        <x:v>Canonical ticket pack</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
         <x:v>FDS_v3.1.19_Canonical_Ticket_Update_Pack_v1.0.md</x:v>
@@ -15250,16 +15285,16 @@
         <x:v>v19 release</x:v>
       </x:c>
       <x:c r="B33" s="146" t="str">
-        <x:v>docs-v3.1.18 remains published</x:v>
+        <x:v>docs-v3.1.19; see CURRENT.md / Release API</x:v>
       </x:c>
       <x:c r="C33" s="146" t="str">
         <x:v>2026-09-17</x:v>
       </x:c>
       <x:c r="D33" s="146" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>Content approved</x:v>
       </x:c>
       <x:c r="E33" s="146" t="str">
-        <x:v>Latest HEAD independent approval pending</x:v>
+        <x:v>PR73 approved/merged. Publication requires finalization approval, Tag and matching Assets. Source notes retain snapshot-time wording.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15288,7 +15323,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.19 · Team Availability Calendar (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.19 · Team Availability Calendar (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>

</xml_diff>